<commit_message>
Leads: 2026-10-10 05:57 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,62 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>The Irish Plumber</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>theirishplumber.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.theirishplumber.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>info@theirishplumber.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>703-924-3100</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Alexandria VA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>plumber Alexandria VA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 06:00 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://www.theirishplumber.com/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>info@theirishplumber.com</t>
@@ -614,6 +613,66 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>KingMade CRC LLC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>kingmadecrc.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.kingmadecrc.com/services/roofing-contractor/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>West Texa</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>kingmadecrc@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(806) 292-8511</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Lubbock TX</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>98</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>roof replacement Lubbock TX</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-10</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-10 06:02 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Valdez Heating and Cooling, LLC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>valdezhvac.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://valdezhvac.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Northwest Arkansas</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>contact@valdezhvac.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(479) 372-3455</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Springdale AR</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>heating and cooling company Springdale AR</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 06:03 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,126 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rock Roof</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>rockroofingde.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://rockroofingde.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Ted Rock</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>tedrockroof@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>302-757-2350</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Wilmington DE</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roof repair company Wilmington DE</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Air Conditioning Repair in Cincinnati, OH</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>gowyomingair.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.gowyomingair.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Brandon Victor</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>wyomingair@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>888-996-4822</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>air conditioning repair Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 06:05 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,66 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Floriano Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>florianosplumbing.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://florianosplumbing.com/locations/danbury-ct.html</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Plumbing Residential</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>dispatch@florianosplumbing.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(888) 809-6756</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Danbury CT</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>plumbing company Danbury CT</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 06:06 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Springfield IL | Coady Roofing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>coadyroofing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://coadyroofing.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Coady Roofing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>mikecoady75@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>217-553-5321</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Springfield IL</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roofing contractor Springfield IL</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 06:08 UTC (cycle 26)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,126 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Good Roofing &amp; Restoration</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>goodroofing.org</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://goodroofing.org/cities/concord/services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Good Roofing</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>wecare@goodroofing.org</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(704) 737-2102</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Concord NC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Metal Roof Survey</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>metalroofsurvey.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.metalroofsurvey.com/metal-roofing-concord/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>For Concord</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@gatormetalroofing.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>866-257-3619</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>96</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Concord NC</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 14:32 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,66 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>True North Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>truenorthroof.net</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://truenorthroof.net/service-areas/thornton</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Hail Damage</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>sasa@truenorthroof.net</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>720-753-4364</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roof repair company Thornton CO</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 14:38 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1158,6 +1158,66 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Carrollton, TX | Carrollton Plumbing</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>carrolltontxplumbing.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://carrolltontxplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Carrollton Homes</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@carrolltontxplumbing.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(831) 666-1222</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Carrollton TX</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>emergency plumber Carrollton TX</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 19:55 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1218,6 +1218,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Shark Construction</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>sharkconstructionllc.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.sharkconstructionllc.com/services/roofing-contractor/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Gutter Repair</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>miguel@sharkconstructionllc.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(540) 809-5299</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roof replacement Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 19:59 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1278,6 +1278,66 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Crowe Services</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>crowehvac.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.crowehvac.com/furnace-repair-maintenance-memphis-tn/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Crowe Services</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>diane@crowehvac.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>901-413-5361</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Memphis TN</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>furnace repair Memphis TN</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 20:05 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1338,6 +1338,62 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Superior Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ocsuperiorplumbing.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://ocsuperiorplumbing.com/services/sewer-line-repair/santa-ana</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>dispatch@ocsuperiorplumbing.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(714) 744-8045</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>94</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>sewer repair Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-10 20:08 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-10.xlsx
+++ b/output/leads_2026-10-10.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1359,7 +1359,6 @@
           <t>https://ocsuperiorplumbing.com/services/sewer-line-repair/santa-ana</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>dispatch@ocsuperiorplumbing.com</t>
@@ -1389,6 +1388,186 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Schoen's Roofing</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>schoensroofing.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.schoensroofing.com/service-areas/iowa-city-ia/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Roof Replacement</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@schoensroofing.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>402-520-7121</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Iowa City IA</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>roofing contractor Iowa City IA</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Unity HVAC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>unityhvac.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://unityhvac.com/service-areas/bethlehem-pa/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Home Improvement</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>info@unityhvac.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(267) 644-9516</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>bbuntingconstruction.com</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>bbuntingconstruction.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://bbuntingconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Jim Murray</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>bryanbunting@southslope.net</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(319) 330-9691</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Iowa City IA</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>88</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>roofing contractor Iowa City IA</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-10-10</t>
         </is>

</xml_diff>